<commit_message>
feat: chuyển sang taxi điện GSM, tách market-research thành 3 skill + research-method, bản 1.2.0
- research-method (nội bộ): phương pháp nguồn/ledger/cache, wb.py, cache.py, form RX
- market-research: đánh giá thị trường taxi điện, khung workbook mới theo R01–R52
- contractor-search, competitor-research: tách từ market-research
- mail-draft: dùng đúng mẫu EX của khách cho CEO/đối ngoại
- project-report: tên GX tiếng Việt; candidate-review: khung tài xế/văn phòng
- bid-review: khung tiêu chí nhà cung cấp GSM, lưu .docx
- doc-compare: từ khoá chính, xác thực nguồn công khai khi được yêu cầu
</commit_message>
<xml_diff>
--- a/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
+++ b/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
@@ -758,7 +758,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>KHUNG BÁO CÁO NGHIÊN CỨU THỊ TRƯỜNG TRẠM SẠC EV</t>
+          <t>KHUNG BÁO CÁO NGHIÊN CỨU THỊ TRƯỜNG TAXI ĐIỆN</t>
         </is>
       </c>
       <c r="B1" s="35" t="n"/>
@@ -824,19 +824,19 @@
     <row r="3" ht="104" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Quy mô thị trường – xe điện</t>
+          <t>Quy mô và cấu trúc thị trường taxi/gọi xe</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>• Tổng số xe điện đang lưu hành.
-• Cơ cấu theo BEV/PHEV và loại xe.
-• Tăng trưởng, doanh số và thị phần tối thiểu 3 năm gần nhất nếu có dữ liệu.</t>
+          <t>• Tổng số chuyến, tổng giá trị đặt xe (GMV) và đội xe đang hoạt động của thị trường taxi và gọi xe ô tô.
+• Cơ cấu theo phân khúc (taxi truyền thống, gọi xe qua app, sân bay, doanh nghiệp) và mức tập trung theo đơn vị vận hành.
+• Số taxi/xe gọi xe chạy điện đang vận hành; tăng trưởng và mùa vụ tối thiểu 3 năm gần nhất nếu có dữ liệu.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nêu rõ định nghĩa xe điện, phạm vi địa lý, kỳ dữ liệu, đơn vị và mẫu số tính thị phần. Ưu tiên cơ quan đăng ký/thống kê; nguồn khác phải được đối chiếu.</t>
+          <t>Nêu rõ ranh giới thị trường, phạm vi địa lý, kỳ dữ liệu và định nghĩa gộp/thuần — GMV không phải doanh thu đơn vị vận hành. Không cộng trùng xe/tài xế chạy nhiều nền tảng. Tách xe đang hoạt động, đã đăng ký, đặt mua và kế hoạch. Ưu tiên cơ quan quản lý vận tải/thống kê; số do nền tảng công bố chỉ đúng cho chính nền tảng đó.</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -863,18 +863,19 @@
     <row r="4" ht="104" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Quy mô thị trường – đội xe dịch vụ</t>
+          <t>Nhu cầu khách hàng và điểm cầu</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>• Số taxi, xe gọi xe, logistics, xe buýt và đội xe dịch vụ chạy điện.
-• Đơn vị vận hành, quy mô đội xe, khu vực hoạt động và kế hoạch mở rộng đã công bố.</t>
+          <t>• Phân khúc khách, mục đích chuyến, mức sẵn lòng chi trả và nhận thức về taxi điện.
+• Điểm phát sinh cầu (sân bay, bến xe, trung tâm thương mại, khu văn phòng, khách sạn), hành lang và khung giờ cao điểm.
+• Quyền đón/trả khách tại các điểm cầu chính và công trình giao thông mới sắp đi vào hoạt động.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Chỉ tính xe đang vận hành khi có bằng chứng. Tách riêng số đang hoạt động, số đặt mua và kế hoạch; không cộng các công bố trùng nhau.</t>
+          <t>Tách sở thích khai báo với hành vi thực tế, lượng khách qua điểm với số chuyến taxi, đánh giá tự chọn với tỷ lệ trên toàn bộ khách. Khớp ranh giới đô thị chức năng và khung giờ. Bản đồ phủ không phải dịch vụ đặt được; quy hoạch không phải hạ tầng đang vận hành.</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -901,18 +902,19 @@
     <row r="5" ht="104" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hạ tầng sạc hiện hữu</t>
+          <t>Bối cảnh vĩ mô và vận hành địa phương</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>• Số trạm và số cổng sạc đang hoạt động theo khu vực/đơn vị vận hành.
-• Vị trí, công suất, chuẩn đầu nối, giá sạc và các trạm đã công bố kế hoạch.</t>
+          <t>• Thu nhập, việc làm, lạm phát và tỷ giá.
+• Du lịch, phương tiện thay thế và biến động đô thị ảnh hưởng tới nhu cầu đi lại.
+• Khí hậu (mưa, ngập, nhiệt), an ninh, an toàn giao thông và gián đoạn lao động ảnh hưởng tới vận hành đội xe.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Định nghĩa rõ trạm và cổng sạc. Tách đang hoạt động, đang xây dựng, kế hoạch và chưa xác minh; ghi ngày khóa dữ liệu và cách xử lý điểm trùng.</t>
+          <t>Dùng dữ liệu địa phương, có kỳ cụ thể; tách thực/danh nghĩa, dự báo/thực tế, quốc gia/địa phương. GDP hay lượng khách du lịch không chứng minh nhu cầu đi taxi. Điều kiện ngập, an ninh tại depot hoặc tuyến cụ thể phải khảo sát riêng.</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -939,18 +941,19 @@
     <row r="6" ht="104" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Tiêu chuẩn và cấu hình sạc</t>
+          <t>Giá cước và mô hình doanh thu</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>• Chuẩn đầu nối AC/DC và dải công suất phổ biến.
-• Số cổng/trụ, phương thức xác thực, giao thức quản lý/roaming và tiêu chuẩn bắt buộc.</t>
+          <t>• Cước mở cửa, cước theo km/phút, phụ phí (sân bay, đêm, cầu đường) và quy định giá cước nếu có.
+• Khuyến mãi, hoa hồng/tỷ lệ thu của nền tảng và cách chia doanh thu với tài xế.
+• Giá hợp đồng doanh nghiệp/sân bay và doanh thu phụ.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Phân biệt yêu cầu pháp lý bắt buộc với cấu hình phổ biến trên thị trường. Dùng quy chuẩn, tài liệu đơn vị vận hành hoặc catalogue có ngày hiệu lực.</t>
+          <t>So sánh trên cùng chuyến mẫu, cùng người trả và cùng cơ sở thuế; tách giá báo trước với cước cuối, khuyến mãi tạm thời với giá thường xuyên. Khoản thu hộ không phải doanh thu đơn vị vận hành. Ghi ngày chụp giá và nguồn (quyết định giá cước, bảng giá chính thức, app).</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -977,18 +980,19 @@
     <row r="7" ht="104" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Đặc tính xe – pin và tiêu thụ</t>
+          <t>Nguồn cung tài xế và thu nhập</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>• Dung lượng pin danh định và khả dụng của các mẫu xe đại diện.
-• Mức tiêu thụ điện (kWh/100 km) và cơ cấu xe mục tiêu.</t>
+          <t>• Nguồn tài xế đủ điều kiện, mô hình hợp tác (nhân viên, đối tác, thuê xe) và kênh tuyển dụng/đào tạo.
+• Thu nhập gộp/thuần, giờ làm, khấu trừ, đặt cọc, thưởng và điều kiện chấm dứt.
+• Rào cản với xe điện (thời gian sạc, đào tạo) và mức lương tham chiếu cho tài xế làm công ăn lương.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Chọn 3–5 mẫu đại diện khi dữ liệu cho phép và giải thích cách chọn. Không tính bình quân nếu chưa có cơ cấu/trọng số; nêu điều kiện thử hoặc nguồn catalogue.</t>
+          <t>Không cộng trùng tài xế chạy nhiều app. Chuẩn hóa theo giờ, thời gian chờ, thời gian sạc và mọi chi phí tài xế tự chịu. Thu nhập quảng cáo tối đa không phải thu nhập thuần điển hình; nhãn thương mại không quyết định tư cách người lao động.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -1015,19 +1019,19 @@
     <row r="8" ht="104" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Đặc tính xe – khả năng sạc</t>
+          <t>Nguồn xe điện và độ phù hợp làm taxi</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>• Công suất sạc AC/DC tối đa.
-• Thời gian sạc theo cùng cửa sổ dung lượng pin, ưu tiên 10–80%.
-• Hạn chế do nhiệt độ hoặc đường cong sạc nếu có.</t>
+          <t>• Các mẫu xe điện được phân phối chính thức, nhà phân phối và giá lăn bánh.
+• Dung lượng pin danh định/khả dụng, tiêu thụ điện (kWh/100 km), quãng đường theo chu kỳ vận hành taxi, công suất sạc AC/DC.
+• Bảo hành khi dùng làm taxi, nguồn cung và thời gian giao xe, triệu hồi, suy giảm pin và giá trị còn lại.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Chỉ so sánh các mẫu xe khi cùng điều kiện đo. Nêu cửa sổ dung lượng pin, nhiệt độ và nguồn; không dùng khái niệm “thời gian sạc trung bình” thiếu điều kiện.</t>
+          <t>Xác minh đúng mẫu/năm/thị trường. Bảo hành xe cá nhân có thể loại trừ taxi. Công suất đỉnh và quãng đường quảng cáo không phải hiệu năng theo chu kỳ taxi; thời gian sạc chỉ so trên cùng cửa sổ pin (ưu tiên 10–80%) và nêu điều kiện đo. Giá rao bán lại không phải giá trị thực hiện được.</t>
         </is>
       </c>
       <c r="D8" s="4" t="n"/>
@@ -1054,19 +1058,19 @@
     <row r="9" ht="104" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Điện thương mại</t>
+          <t>Sạc cho đội xe</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>• Đơn vị điện lực, biểu giá và nhóm khách hàng áp dụng.
-• Giá điện, thuế/phí, phí công suất và giờ cao–thấp điểm.
-• Quy trình đấu nối công khai.</t>
+          <t>• Phương án sạc cho đội xe: sạc tại depot, sạc cơ hội trong ca, sạc công cộng, đổi pin — thời gian dừng và năng lượng cần theo ca.
+• Mạng sạc công cộng dùng làm dự phòng: số điểm và số cổng đang hoạt động, công suất khả dụng, chuẩn đầu nối, giá sạc.
+• Chuẩn đầu nối/giao thức phổ biến và độ tương thích với mẫu xe mục tiêu.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Dùng biểu giá của cơ quan quản lý/điện lực, ghi ngày hiệu lực, điện áp, tiền tệ và thuế. Công suất và chi phí tại địa điểm cụ thể phải tách thành Chưa xác minh.</t>
+          <t>Tách điểm sạc, cổng sạc và công suất đồng thời; đã nghiệm thu không phải dùng được, trực tuyến không phải sạc thành công. Giá điện không phải giá sạc công cộng. Không đưa ra thiết kế kỹ thuật hay số bộ sạc cho đội xe từ benchmark chưa đủ.</t>
         </is>
       </c>
       <c r="D9" s="4" t="n"/>
@@ -1093,18 +1097,19 @@
     <row r="10" ht="104" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Hạ tầng thanh toán</t>
+          <t>Điện thương mại và đấu nối depot</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>• Phương thức thanh toán phổ biến và phương thức dùng tại trạm sạc.
-• Nhà cung cấp, phí công khai, thời gian đối soát, hoàn tiền và khả năng tích hợp.</t>
+          <t>• Đơn vị điện lực, biểu giá và nhóm khách hàng áp dụng cho depot sạc.
+• Giá điện năng, phí công suất, giờ cao–thấp điểm, thuế/phí.
+• Quy trình, thời gian và phân bổ chi phí đấu nối công khai; độ tin cậy cấp điện và phương án dự phòng.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nêu rõ phạm vi áp dụng và điều kiện của nhà cung cấp. Phí hoặc tỷ lệ giao dịch thành công không công khai phải ghi Chưa xác minh, không tự ước đoán.</t>
+          <t>Dùng biểu giá của cơ quan quản lý/điện lực, ghi ngày hiệu lực, điện áp, tiền tệ và thuế. Trạm biến áp gần không chứng minh còn công suất; công suất và chi phí đấu nối tại depot cụ thể phải tách thành Chưa xác minh cho đến khi điện lực xác nhận.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
@@ -1131,18 +1136,19 @@
     <row r="11" ht="104" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Hạ tầng viễn thông</t>
+          <t>Depot, bãi đỗ và mặt bằng</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>• Mức phủ 4G/5G và cáp quang tại khu vực mục tiêu.
-• Nhà mạng, phương án kết nối chính/dự phòng và điều kiện dịch vụ công khai.</t>
+          <t>• Loại mặt bằng phù hợp làm depot (bãi đỗ, kho, đất khu công nghiệp) và tình trạng sẵn có tại khu vực mục tiêu.
+• Giá thuê, thời hạn, quyền sử dụng và mục đích sử dụng được phép.
+• Đường ra vào, nguồn điện, hạn chế môi trường/quy hoạch và nghĩa vụ hoàn trả mặt bằng.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bản đồ phủ sóng chỉ dùng ở cấp khu vực. Băng thông, độ trễ, độ ổn định và thời gian khắc phục tại địa điểm phải được nhà mạng hoặc khảo sát xác nhận.</t>
+          <t>Tin rao không phải mặt bằng đã xác minh sẵn có hay được phép sử dụng. Nguồn điện gần không phải công suất tại mặt bằng. Nghiên cứu bàn giấy không thay khảo sát hiện trường; điều kiện tại địa điểm cụ thể ghi Chưa xác minh.</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -1169,18 +1175,19 @@
     <row r="12" ht="104" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Điều kiện tự nhiên</t>
+          <t>Bảo dưỡng, phụ tùng và cứu hộ</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>• Nhiệt độ, độ ẩm, mưa, ngập, sét, bụi/ăn mòn và hiện tượng cực đoan.
-• Tác động đến thiết bị, nền trạm, thoát nước, che chắn và thi công.</t>
+          <t>• Mạng lưới xưởng dịch vụ cho đúng mẫu xe mục tiêu và kỹ thuật viên có chứng chỉ điện cao áp.
+• Nguồn phụ tùng, tồn kho, giá dịch vụ và thời gian xe nằm xưởng.
+• Cứu hộ xe điện, kênh xử lý pin thay thế và tái chế.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Nêu chu kỳ dữ liệu, cực trị, vị trí trạm đo/bản đồ và phạm vi địa lý. Điều kiện thoát nước hoặc lịch sử ngập tại địa điểm phải khảo sát riêng.</t>
+          <t>Có trong catalogue không phải có tồn kho. Thời gian sửa không phải tổng thời gian dừng xe. Kiểm tra loại trừ bảo hành với xe taxi và sửa chữa bên thứ ba; tách pin thay thế với tái sử dụng/tái chế đủ điều kiện.</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
@@ -1207,18 +1214,19 @@
     <row r="13" ht="104" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>An ninh và an toàn khu vực</t>
+          <t>Thanh toán, kết nối và dữ liệu</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>• Rủi ro trộm cắp, phá hoại, gian lận và an toàn giao thông.
-• Các biện pháp bảo vệ, chiếu sáng, camera, kiểm soát ra/vào và phản ứng sự cố.</t>
+          <t>• Phương thức thanh toán phổ biến cho chuyến xe (tiền mặt, thẻ, ví điện tử, mobile money) và đơn vị được cấp phép.
+• Phí, thời gian đối soát, hoàn tiền và khả năng tích hợp API.
+• Phủ sóng 4G/5G phục vụ app và điều phối; quy định lưu trữ dữ liệu và chuyển dữ liệu ra nước ngoài.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Chỉ sử dụng thống kê sự cố, bản đồ rủi ro hoặc nguồn đáng tin cậy. Không khái quát hóa toàn thành phố; điều kiện tại địa điểm phải được khảo sát.</t>
+          <t>Tỷ lệ sử dụng toàn quốc và bản đồ phủ sóng có thể che vùng bị loại trừ. Tài liệu API không phải tích hợp đã thử; khả dụng kỹ thuật không phải được phép. Phí hoặc tỷ lệ giao dịch thành công không công khai phải ghi Chưa xác minh, không tự ước đoán.</t>
         </is>
       </c>
       <c r="D13" s="4" t="n"/>
@@ -1243,21 +1251,21 @@
       <c r="W13" s="1" t="n"/>
     </row>
     <row r="14" ht="104" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Kết luận tổng quan và nhu cầu sạc</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chi phí, TCO và kinh tế đơn vị</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>• 3–5 phát hiện ảnh hưởng trực tiếp đến nhu cầu và triển khai.
-• Khu vực ưu tiên, cấu hình sạc sơ bộ và nhu cầu điện theo giai đoạn.
-• Dữ liệu còn thiếu và bước xác minh tiếp theo.</t>
+          <t>• Phạm vi kinh tế được định nghĩa: giá xe, chi phí thiết lập, năng lượng, bảo dưỡng, bảo hiểm, tài chính, giá trị còn lại.
+• Doanh thu và năng suất tham chiếu (chuyến/xe/ngày, tỷ lệ km có khách).
+• Điểm hòa vốn minh họa, độ nhạy và biến động chi phí.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tách rõ dữ liệu đã xác minh, ước tính và chưa xác minh. Mọi phép tính có công thức/giả định; không kết luận một địa điểm sẵn sàng nếu thiếu quyền sử dụng đất, điện và pháp lý.</t>
+          <t>Khớp km có khách/tổng km, cơ sở thuế và kỳ hạn. Không tính trùng tổn hao sạc hoặc tính cả giá mua, khấu hao và gốc thuê. Mọi phép tính ghi công thức, đầu vào và giả định (Ước tính); có giới hạn công suất; không kết luận lợi nhuận của công ty.</t>
         </is>
       </c>
       <c r="D14" s="4" t="n"/>
@@ -1281,17 +1289,27 @@
       <c r="V14" s="1" t="n"/>
       <c r="W14" s="1" t="n"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>BẢNG 2 — PHÁP LÝ, GIẤY PHÉP VÀ CÁC THỦ TỤC CÓ THỂ LÀM CHẬM DỰ ÁN</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="20" t="n"/>
+    <row r="15" ht="104" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chất lượng dịch vụ và an toàn</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>• Cam kết dịch vụ và chỉ số chất lượng công khai (tỷ lệ nhận/hủy chuyến, thời gian đón, đánh giá khách).
+• Yêu cầu an toàn với hành khách, tài xế và xe điện; cơ chế xử lý sự cố, khiếu nại và bảo hiểm.
+• Sự cố đã được xác minh trên thị trường và thay đổi quy định sau đó.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Cam kết không phải kết quả. Tách yêu cầu bắt buộc với tự nguyện. So tỷ lệ trên cùng mẫu số và mức độ nghiêm trọng; không kết luận nhân quả từ thông tin ban đầu. Thống kê sự cố chỉ dùng đúng phạm vi địa lý của nó.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
       <c r="G15" s="1" t="n"/>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
@@ -1310,32 +1328,27 @@
       <c r="V15" s="1" t="n"/>
       <c r="W15" s="1" t="n"/>
     </row>
-    <row r="16" ht="56" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Thủ tục</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Cơ quan xử lý</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Căn cứ và hồ sơ chính</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Thời gian xử lý</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Phí/lệ phí</t>
-        </is>
-      </c>
+    <row r="16" ht="104" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Kết luận tổng quan và tiềm năng thị trường</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>• 3–5 phát hiện ảnh hưởng trực tiếp đến nhu cầu và vận hành đội taxi điện.
+• Khu vực/điểm cầu ưu tiên, quy mô đội xe và nhu cầu sạc/điện sơ bộ theo giai đoạn.
+• Dữ liệu còn thiếu và bước xác minh tiếp theo.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Tách rõ dữ liệu đã xác minh, ước tính và chưa xác minh. Mọi phép tính có công thức/giả định; không kết luận thị trường sẵn sàng khai trương nếu thiếu xác nhận về giấy phép vận tải, nguồn xe, depot/điện và chi phí.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
       <c r="G16" s="1" t="n"/>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
@@ -1354,33 +1367,17 @@
       <c r="V16" s="1" t="n"/>
       <c r="W16" s="1" t="n"/>
     </row>
-    <row r="17" ht="122.75" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Thành lập pháp nhân</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Tên pháp lý của cơ quan có thẩm quyền và URL/cổng chính thức. Nếu chưa xác định được, ghi Chưa xác minh.</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Tên/số văn bản, điều khoản, ngày hiệu lực; 
-Liệt kê các điều kiện, danh sách hồ sơ và thứ tự thực hiện.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Thời hạn công bố hoặc kinh nghiệm thực tế có nguồn. Nếu không có dữ liệu phù hợp, ghi Chưa xác minh; không tự tạo khoảng thời gian.</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Phí/lệ phí chính thức và căn cứ. Chi phí tư vấn, dịch vụ hoặc bên thứ ba phải tách riêng; không ước tính nếu chưa có nguồn/báo giá.</t>
-        </is>
-      </c>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>BẢNG 2 — PHÁP LÝ, GIẤY PHÉP VÀ CÁC THỦ TỤC CÓ THỂ LÀM CHẬM DỰ ÁN</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="20" t="n"/>
       <c r="G17" s="1" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
@@ -1399,31 +1396,30 @@
       <c r="V17" s="1" t="n"/>
       <c r="W17" s="1" t="n"/>
     </row>
-    <row r="18" ht="122.75" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Giấy phép hoạt động doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Tên pháp lý của cơ quan có thẩm quyền và URL/cổng chính thức. Nếu chưa xác định được, ghi Chưa xác minh.</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Tên/số văn bản, điều khoản, ngày hiệu lực; 
-Liệt kê các điều kiện, danh sách hồ sơ và thứ tự thực hiện.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Thời hạn công bố hoặc kinh nghiệm thực tế có nguồn. Nếu không có dữ liệu phù hợp, ghi Chưa xác minh; không tự tạo khoảng thời gian.</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Phí/lệ phí chính thức và căn cứ. Chi phí tư vấn, dịch vụ hoặc bên thứ ba phải tách riêng; không ước tính nếu chưa có nguồn/báo giá.</t>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Thủ tục</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Cơ quan xử lý</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Căn cứ và hồ sơ chính</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Thời gian xử lý</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Phí/lệ phí</t>
         </is>
       </c>
       <c r="G18" s="1" t="n"/>
@@ -1447,7 +1443,7 @@
     <row r="19" ht="122.75" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Giấy phép bán điện hoặc cung cấp dịch vụ sạc</t>
+          <t>Thành lập pháp nhân và đầu tư nước ngoài</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1492,7 +1488,7 @@
     <row r="20" ht="122.75" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Giấy phép xây dựng hoặc lắp đặt</t>
+          <t>Giấy phép kinh doanh vận tải taxi</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1537,7 +1533,7 @@
     <row r="21" ht="122.75" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Chấp thuận đấu nối và cấp điện</t>
+          <t>Điều kiện tài xế và giấy phép hành nghề</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1582,7 +1578,7 @@
     <row r="22" ht="122.75" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PCCC, an ninh và an toàn</t>
+          <t>Nền tảng gọi xe và điều phối</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1627,7 +1623,7 @@
     <row r="23" ht="122.75" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Môi trường, quy hoạch hoặc đào đường</t>
+          <t>Nhập khẩu, đồng bộ và đăng kiểm xe</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1672,7 +1668,7 @@
     <row r="24" ht="122.75" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Bảo vệ dữ liệu cá nhân và an ninh mạng</t>
+          <t>Thuế, hải quan và ưu đãi xe điện</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1717,7 +1713,7 @@
     <row r="25" ht="122.75" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Thanh toán, hóa đơn và thuế</t>
+          <t>Depot và sạc: xây dựng, đấu nối, PCCC</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1759,17 +1755,33 @@
       <c r="V25" s="1" t="n"/>
       <c r="W25" s="1" t="n"/>
     </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>BẢNG 3 — ĐÁNH GIÁ SƠ BỘ NHÀ THẦU, NHÀ CUNG CẤP VÀ ĐỐI TÁC ĐỊA PHƯƠNG</t>
-        </is>
-      </c>
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
+    <row r="26" ht="122.75" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Lao động và bảo hiểm tài xế</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Tên pháp lý của cơ quan có thẩm quyền và URL/cổng chính thức. Nếu chưa xác định được, ghi Chưa xác minh.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Tên/số văn bản, điều khoản, ngày hiệu lực; 
+Liệt kê các điều kiện, danh sách hồ sơ và thứ tự thực hiện.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Thời hạn công bố hoặc kinh nghiệm thực tế có nguồn. Nếu không có dữ liệu phù hợp, ghi Chưa xác minh; không tự tạo khoảng thời gian.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Phí/lệ phí chính thức và căn cứ. Chi phí tư vấn, dịch vụ hoặc bên thứ ba phải tách riêng; không ước tính nếu chưa có nguồn/báo giá.</t>
+        </is>
+      </c>
       <c r="G26" s="1" t="n"/>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="1" t="n"/>
@@ -1788,35 +1800,31 @@
       <c r="V26" s="1" t="n"/>
       <c r="W26" s="1" t="n"/>
     </row>
-    <row r="27" ht="56" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Nhóm đối tác</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Đơn vị và liên hệ</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Phạm vi cung cấp</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Pháp lý/chứng nhận</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Kinh nghiệm liên quan</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Năng lực và hiện diện địa phương</t>
+    <row r="27" ht="122.75" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Bảo vệ dữ liệu cá nhân, thanh toán và hóa đơn</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Tên pháp lý của cơ quan có thẩm quyền và URL/cổng chính thức. Nếu chưa xác định được, ghi Chưa xác minh.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Tên/số văn bản, điều khoản, ngày hiệu lực; 
+Liệt kê các điều kiện, danh sách hồ sơ và thứ tự thực hiện.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Thời hạn công bố hoặc kinh nghiệm thực tế có nguồn. Nếu không có dữ liệu phù hợp, ghi Chưa xác minh; không tự tạo khoảng thời gian.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Phí/lệ phí chính thức và căn cứ. Chi phí tư vấn, dịch vụ hoặc bên thứ ba phải tách riêng; không ước tính nếu chưa có nguồn/báo giá.</t>
         </is>
       </c>
       <c r="G27" s="1" t="n"/>
@@ -1837,40 +1845,17 @@
       <c r="V27" s="1" t="n"/>
       <c r="W27" s="1" t="n"/>
     </row>
-    <row r="28" ht="133.25" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Nhà thầu xây dựng</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (§6.2 SKILL.md) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Turnkey (Thiết kế, xây dựng dân dụng, điện, xin phép, thử nghiệm và nghiệm thu.)</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.
-Bắt buộc: mã ngành kinh doanh chính (từ cổng đăng ký kinh doanh quốc gia) và năm thành lập, kèm nguồn tra cứu.</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.
-Vai trò chuỗi cung ứng ghi tại Bảng 3B: Tổng thầu turnkey / Cấp 1 chuyên ngành / Trung gian-Đại lý (Cấp 2) / Chưa xác định. Chỉ Tổng thầu turnkey mới vào danh sách 'Nhà thầu phù hợp sơ bộ'. Turnkey bắt buộc có ≥1 bằng chứng độc lập; hồ sơ năng lực tự công bố không đủ. Không loại đơn vị chỉ vì website có chữ đại lý/phân phối — nhiều tổng thầu vừa thi công vừa phân phối thiết bị; chỉ loại khi thiếu bằng chứng tự thi công.</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.
-Kèm kiểm tra LinkedIn/trang mạng xã hội công ty: mô tả có nêu rõ thi công/xây lắp/tổng thầu/EPC hay không.</t>
-        </is>
-      </c>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>BẢNG 3 — ĐÁNH GIÁ SƠ BỘ NHÀ THẦU, NHÀ CUNG CẤP VÀ ĐỐI TÁC ĐỊA PHƯƠNG</t>
+        </is>
+      </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
       <c r="G28" s="1" t="n"/>
       <c r="H28" s="1" t="n"/>
       <c r="I28" s="1" t="n"/>
@@ -1889,35 +1874,35 @@
       <c r="V28" s="1" t="n"/>
       <c r="W28" s="1" t="n"/>
     </row>
-    <row r="29" ht="133.25" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Đơn vị vận hành trạm/CPO (Đối thủ kinh doanh)</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Nền tảng quản lý, vận hành, roaming, chăm sóc khách hàng và thanh toán.</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.</t>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm đối tác</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Đơn vị và liên hệ</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Phạm vi cung cấp</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Pháp lý/chứng nhận</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm liên quan</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Năng lực và hiện diện địa phương</t>
         </is>
       </c>
       <c r="G29" s="1" t="n"/>
@@ -1941,32 +1926,35 @@
     <row r="30" ht="133.25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Đơn vị logistics và hải quan</t>
+          <t>Nhà thầu xây depot và lắp sạc</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
+          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (F1–F10, skill contractor-search) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Vận tải, thông quan, mã hàng, thuế/phí, giao hàng tới địa điểm và bảo hiểm hàng hóa.</t>
+          <t>Turnkey (Thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc cho đội xe, xin phép, thử nghiệm và nghiệm thu.)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.</t>
+          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.
+Bắt buộc: mã ngành kinh doanh chính (từ cổng đăng ký kinh doanh quốc gia) và năm thành lập, kèm nguồn tra cứu.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.</t>
+          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.
+Vai trò chuỗi cung ứng ghi tại Bảng 3B: Tổng thầu turnkey / Cấp 1 chuyên ngành / Trung gian-Đại lý (Cấp 2) / Chưa xác định. Chỉ Tổng thầu turnkey mới vào danh sách 'Nhà thầu phù hợp sơ bộ'. Turnkey bắt buộc có ≥1 bằng chứng độc lập; hồ sơ năng lực tự công bố không đủ. Không loại đơn vị chỉ vì website có chữ đại lý/phân phối — nhiều tổng thầu vừa thi công vừa phân phối thiết bị; chỉ loại khi thiếu bằng chứng tự thi công.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.</t>
+          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.
+Kèm kiểm tra LinkedIn/trang mạng xã hội công ty: mô tả có nêu rõ thi công/xây lắp/tổng thầu/EPC hay không.</t>
         </is>
       </c>
       <c r="G30" s="1" t="n"/>
@@ -1990,7 +1978,7 @@
     <row r="31" ht="133.25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Công ty luật/tư vấn giấy phép</t>
+          <t>Nguồn xe – OEM/nhà phân phối</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2000,7 +1988,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Pháp nhân, giấy phép, năng lượng, xây dựng, dữ liệu, lao động và thuế.</t>
+          <t>Mẫu xe phân phối chính thức, giá lăn bánh, bảo hành khi dùng làm taxi, thời gian giao xe, phụ tùng và hỗ trợ kỹ thuật tại địa phương.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2039,7 +2027,7 @@
     <row r="32" ht="133.25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Đơn vị viễn thông</t>
+          <t>Tài chính, thuê xe và bảo hiểm</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2049,7 +2037,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>4G/5G, cáp quang, mạng riêng, dự phòng, giám sát và cam kết dịch vụ.</t>
+          <t>Cho vay/thuê tài chính xe taxi, điều kiện, phí và lãi suất quy đổi; bảo hiểm xe, trách nhiệm hành khách, pin/xe điện, loại trừ và bồi thường.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2088,7 +2076,7 @@
     <row r="33" ht="133.25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Ngân hàng/đơn vị thanh toán</t>
+          <t>Bảo dưỡng, sửa chữa</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2098,7 +2086,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản, cổng thanh toán, thiết bị, đối soát, hoàn tiền và tích hợp.</t>
+          <t>Xưởng dịch vụ đúng mẫu xe, kỹ thuật viên điện cao áp, phụ tùng, cứu hộ xe điện, giá dịch vụ và thời gian xe nằm xưởng.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2137,7 +2125,7 @@
     <row r="34" ht="133.25" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Bảo hiểm</t>
+          <t>Công nghệ gọi xe và điều phối</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2147,7 +2135,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Tài sản, trách nhiệm, xây dựng/lắp đặt, gián đoạn kinh doanh và rủi ro mạng.</t>
+          <t>Ứng dụng đặt xe, điều phối, công cụ tài xế/đội xe, API và quyền dữ liệu, bảo mật, phí đầy đủ và hỗ trợ tại chỗ.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2183,17 +2171,37 @@
       <c r="V34" s="1" t="n"/>
       <c r="W34" s="1" t="n"/>
     </row>
-    <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>BẢNG 4 — RỦI RO VÀ KẾ HOẠCH XÁC MINH</t>
-        </is>
-      </c>
-      <c r="B35" s="35" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="35" t="n"/>
-      <c r="E35" s="35" t="n"/>
-      <c r="F35" s="35" t="n"/>
+    <row r="35" ht="133.25" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Dịch vụ đội xe hằng ngày</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Vệ sinh xe, bãi đỗ và chuẩn bị xe, vật tư tiêu hao, năng lực giờ cao điểm, giấy phép nước/chất thải và phương án dự phòng.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.</t>
+        </is>
+      </c>
       <c r="G35" s="1" t="n"/>
       <c r="H35" s="1" t="n"/>
       <c r="I35" s="1" t="n"/>
@@ -2212,35 +2220,35 @@
       <c r="V35" s="1" t="n"/>
       <c r="W35" s="1" t="n"/>
     </row>
-    <row r="36" ht="56" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>Nhóm rủi ro</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Rủi ro cụ thể (Nguyên nhân – Sự kiện – Hậu quả)</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Khả năng xảy ra</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>Tác động tiến độ</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>Tác động chi phí</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Khả năng kiểm soát</t>
+    <row r="36" ht="133.25" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Luật, thuế và tư vấn</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Pháp nhân, giấy phép vận tải, thuế, kế toán/kiểm toán, lương và lao động, mở tài khoản ngân hàng, dữ liệu.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.</t>
         </is>
       </c>
       <c r="G36" s="1" t="n"/>
@@ -2261,35 +2269,35 @@
       <c r="V36" s="1" t="n"/>
       <c r="W36" s="1" t="n"/>
     </row>
-    <row r="37" ht="117.25" customHeight="1">
+    <row r="37" ht="133.25" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Điện và lưới điện</t>
+          <t>Tuyển dụng và đào tạo tài xế</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Thiếu công suất, chậm đấu nối/trạm biến áp, biểu giá, mất điện, chất lượng điện hoặc thiếu xác nhận của điện lực.</t>
+          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Cao / Trung bình / Thấp / Chưa đủ dữ liệu. Chỉ chọn mức khi có bằng chứng hoặc dữ liệu dự án và phải nêu căn cứ.</t>
+          <t>Nguồn tài xế đủ điều kiện, sàng lọc lý lịch, đào tạo lái xe điện và dịch vụ, hỗ trợ cấp giấy phép hành nghề, phí dịch vụ.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Nêu số ngày/tuần khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu và giải thích.</t>
+          <t>Chỉ ghi đăng ký, giấy phép hoặc chứng nhận khi có tên/số, đơn vị cấp, hiệu lực và nguồn. Không tìm thấy phải ghi Chưa xác minh.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Nêu khoảng tiền hoặc % ngân sách khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Cao / Trung bình / Thấp. Nêu biện pháp, người chịu trách nhiệm và nguồn lực; kế hoạch chưa xác nhận phải ghi rõ.</t>
+          <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Nêu văn phòng, đội ngũ, kho/phụ tùng, vùng phục vụ hoặc năng lực được công bố. Năng lực thực tế chưa công khai phải ghi Chưa xác minh.</t>
         </is>
       </c>
       <c r="G37" s="1" t="n"/>
@@ -2310,37 +2318,17 @@
       <c r="V37" s="1" t="n"/>
       <c r="W37" s="1" t="n"/>
     </row>
-    <row r="38" ht="117.25" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Pháp lý và giấy phép</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Giấy phép chưa rõ, hồ sơ thiếu, thay đổi quy định, thủ tục nối tiếp hoặc nội dung cần giải thích pháp lý.</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Cao / Trung bình / Thấp / Chưa đủ dữ liệu. Chỉ chọn mức khi có bằng chứng hoặc dữ liệu dự án và phải nêu căn cứ.</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Nêu số ngày/tuần khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu và giải thích.</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Nêu khoảng tiền hoặc % ngân sách khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Cao / Trung bình / Thấp. Nêu biện pháp, người chịu trách nhiệm và nguồn lực; kế hoạch chưa xác nhận phải ghi rõ.</t>
-        </is>
-      </c>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>BẢNG 4 — RỦI RO VÀ KẾ HOẠCH XÁC MINH</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="35" t="n"/>
+      <c r="E38" s="35" t="n"/>
+      <c r="F38" s="35" t="n"/>
       <c r="G38" s="1" t="n"/>
       <c r="H38" s="1" t="n"/>
       <c r="I38" s="1" t="n"/>
@@ -2359,36 +2347,35 @@
       <c r="V38" s="1" t="n"/>
       <c r="W38" s="1" t="n"/>
     </row>
-    <row r="39" ht="117.25" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Nhà thầu</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Thiếu năng lực/nhân lực, phạm vi công việc không rõ, an toàn/chất lượng, tiến độ, bảo lãnh hoặc tranh chấp.
-Văn hoá &amp; hành vi hợp tác giữa nhà thầu và chủ đầu tư</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Cao / Trung bình / Thấp / Chưa đủ dữ liệu. Chỉ chọn mức khi có bằng chứng hoặc dữ liệu dự án và phải nêu căn cứ.</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Nêu số ngày/tuần khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu và giải thích.</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Nêu khoảng tiền hoặc % ngân sách khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu.</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Cao / Trung bình / Thấp. Nêu biện pháp, người chịu trách nhiệm và nguồn lực; kế hoạch chưa xác nhận phải ghi rõ.</t>
+    <row r="39" ht="56" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm rủi ro</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Rủi ro cụ thể (Nguyên nhân – Sự kiện – Hậu quả)</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Khả năng xảy ra</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tác động tiến độ</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Tác động chi phí</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Khả năng kiểm soát</t>
         </is>
       </c>
       <c r="G39" s="1" t="n"/>
@@ -2412,12 +2399,12 @@
     <row r="40" ht="117.25" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Nhà cung cấp và thiết bị</t>
+          <t>Pháp lý vận tải và giấy phép</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Không tương thích với xe/lưới/phần mềm, thiếu chứng nhận, giao hàng chậm, bảo hành, phụ tùng hoặc hỗ trợ địa phương.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Giấy phép taxi/nền tảng chưa rõ, hạn ngạch xe, quyền đón khách bị giới hạn, hồ sơ thiếu, thay đổi quy định, thủ tục nối tiếp hoặc nội dung cần giải thích pháp lý.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2461,12 +2448,12 @@
     <row r="41" ht="117.25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Logistics và nhập khẩu</t>
+          <t>Nguồn xe và nhập khẩu</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Mã hàng/chứng từ, vận tải, hải quan, thuế/phí, hàng quá khổ, lưu container, hư hỏng hoặc giao địa điểm.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Mẫu xe chưa được phê duyệt/đăng kiểm, giao xe chậm, thuế nhập khẩu hoặc ưu đãi thay đổi, bảo hành không áp dụng cho taxi, thiếu phụ tùng, vận chuyển pin.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2510,12 +2497,12 @@
     <row r="42" ht="117.25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Tỷ giá và giá vật tư</t>
+          <t>Tài xế và lao động</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Biến động tỷ giá, đồng/thép/thiết bị, lạm phát, thời hạn báo giá và điều khoản điều chỉnh giá.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Thiếu tài xế đủ điều kiện, tỷ lệ nghỉ việc cao, tranh chấp tư cách người lao động, chi phí bảo hiểm bắt buộc, đào tạo lái xe điện hoặc đình công.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2559,12 +2546,12 @@
     <row r="43" ht="117.25" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Công nghệ và thanh toán</t>
+          <t>Sạc và điện cho đội xe</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Kết nối, phần mềm quản lý, giao thức/API, lỗi thanh toán/đối soát, an ninh mạng và bảo vệ dữ liệu.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Thiếu công suất tại depot, chậm đấu nối/trạm biến áp, biểu giá, mất điện, sạc công cộng thiếu hoặc phải xếp hàng, xe chờ sạc làm giảm số chuyến.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2608,12 +2595,12 @@
     <row r="44" ht="117.25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>An ninh và khí hậu</t>
+          <t>Cạnh tranh và giá cước</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Trộm cắp, phá hoại, tai nạn, ngập, sét, nhiệt, bụi/ăn mòn hoặc gián đoạn hoạt động tại địa điểm.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Đối thủ trợ giá/khuyến mãi, cuộc chiến giá cước, trần/sàn giá theo quy định, hợp đồng độc quyền sân bay/doanh nghiệp, tài xế bị lôi kéo.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2657,12 +2644,12 @@
     <row r="45" ht="117.25" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Vận hành và bảo trì</t>
+          <t>Vận hành, an toàn và sự cố</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Thiếu quy trình/nhân sự/phụ tùng, thời gian ngừng hoạt động, sửa chữa chậm, quá tải hoặc trải nghiệm khách hàng kém.</t>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Tai nạn, sự cố an toàn hành khách, cháy pin, trộm cắp/phá hoại tại depot, ngập, xe nằm xưởng lâu, trải nghiệm khách hàng kém.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2703,30 +2690,35 @@
       <c r="V45" s="1" t="n"/>
       <c r="W45" s="1" t="n"/>
     </row>
-    <row r="46" ht="42" customHeight="1">
-      <c r="A46" s="23" t="inlineStr">
-        <is>
-          <t>Tổng kết</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Nêu rủi ro có khả năng cao nhất hoặc chưa đủ dữ liệu.</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Nêu khoảng chậm khi có cơ sở; nếu chưa có, lập kế hoạch thu thập dữ liệu.</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Nêu khoảng chi phí khi có cơ sở; tránh cộng trùng dự phòng.</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Biện pháp, người chịu trách nhiệm và điều kiện hoàn thành.</t>
+    <row r="46" ht="117.25" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Tỷ giá và chi phí</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: Biến động tỷ giá, giá xe/pin, lãi suất tài chính, lạm phát, giá điện, thời hạn báo giá và điều khoản điều chỉnh giá.</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Cao / Trung bình / Thấp / Chưa đủ dữ liệu. Chỉ chọn mức khi có bằng chứng hoặc dữ liệu dự án và phải nêu căn cứ.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Nêu số ngày/tuần khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu và giải thích.</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Nêu khoảng tiền hoặc % ngân sách khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Cao / Trung bình / Thấp. Nêu biện pháp, người chịu trách nhiệm và nguồn lực; kế hoạch chưa xác nhận phải ghi rõ.</t>
         </is>
       </c>
       <c r="G46" s="1" t="n"/>
@@ -2747,21 +2739,37 @@
       <c r="V46" s="1" t="n"/>
       <c r="W46" s="1" t="n"/>
     </row>
-    <row r="47" ht="45.25" customHeight="1">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>KẾT LUẬN PHÁP LÝ</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Mỗi kết quả phải gồm: kết luận | trạng thái | nguồn và ngày | giới hạn | hành động xác minh</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
+    <row r="47" ht="117.25" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Công nghệ, thanh toán và dữ liệu</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Viết theo cấu trúc Nguyên nhân – Sự kiện – Hậu quả. Phạm vi tối thiểu: App/điều phối gián đoạn, lỗi thanh toán/đối soát, gian lận, chargeback, an ninh mạng, bảo vệ dữ liệu cá nhân và chuyển dữ liệu ra nước ngoài.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Cao / Trung bình / Thấp / Chưa đủ dữ liệu. Chỉ chọn mức khi có bằng chứng hoặc dữ liệu dự án và phải nêu căn cứ.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Nêu số ngày/tuần khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu và giải thích.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Nêu khoảng tiền hoặc % ngân sách khi có cơ sở; nếu chưa thể định lượng, dùng Cao/Trung bình/Thấp hoặc Chưa đủ dữ liệu.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Cao / Trung bình / Thấp. Nêu biện pháp, người chịu trách nhiệm và nguồn lực; kế hoạch chưa xác nhận phải ghi rõ.</t>
+        </is>
+      </c>
       <c r="G47" s="1" t="n"/>
       <c r="H47" s="1" t="n"/>
       <c r="I47" s="1" t="n"/>
@@ -2780,21 +2788,32 @@
       <c r="V47" s="1" t="n"/>
       <c r="W47" s="1" t="n"/>
     </row>
-    <row r="48" ht="77.25" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Thủ tục có thời gian xử lý dài nhất</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Nêu thủ tục có thời hạn dài nhất và nguồn; tách thời hạn chính thức với kinh nghiệm thực tế. Nếu không đủ dữ liệu so sánh, ghi Chưa xác minh.</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
+    <row r="48" ht="42" customHeight="1">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>Tổng kết</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Nêu rủi ro có khả năng cao nhất hoặc chưa đủ dữ liệu.</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Nêu khoảng chậm khi có cơ sở; nếu chưa có, lập kế hoạch thu thập dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Nêu khoảng chi phí khi có cơ sở; tránh cộng trùng dự phòng.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Biện pháp, người chịu trách nhiệm và điều kiện hoàn thành.</t>
+        </is>
+      </c>
       <c r="G48" s="1" t="n"/>
       <c r="H48" s="1" t="n"/>
       <c r="I48" s="1" t="n"/>
@@ -2813,15 +2832,15 @@
       <c r="V48" s="1" t="n"/>
       <c r="W48" s="1" t="n"/>
     </row>
-    <row r="49" ht="77.25" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Nội dung pháp lý chưa có kết luận chính thức</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Nêu câu hỏi chưa có kết luận, văn bản đã tìm, điểm mâu thuẫn, cơ quan/luật sư cần hỏi, tài liệu và thời hạn xác minh.</t>
+    <row r="49" ht="45.25" customHeight="1">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>KẾT LUẬN PHÁP LÝ</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Mỗi kết quả phải gồm: kết luận | trạng thái | nguồn và ngày | giới hạn | hành động xác minh</t>
         </is>
       </c>
       <c r="C49" s="4" t="n"/>
@@ -2849,12 +2868,12 @@
     <row r="50" ht="77.25" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Thời gian dự phòng cần cộng thêm cho pháp lý</t>
+          <t>Thủ tục có thời gian xử lý dài nhất</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Chỉ đưa khoảng dự phòng khi có thời hạn, trường hợp tham chiếu hoặc dữ liệu dự án. Nếu là giả định kế hoạch, phải ghi rõ phương pháp và cơ sở.</t>
+          <t>Nêu thủ tục có thời hạn dài nhất trước khi đội xe được khai thác, kèm nguồn; tách thời hạn chính thức với kinh nghiệm thực tế. Nếu không đủ dữ liệu so sánh, ghi Chưa xác minh.</t>
         </is>
       </c>
       <c r="C50" s="4" t="n"/>
@@ -2879,15 +2898,15 @@
       <c r="V50" s="1" t="n"/>
       <c r="W50" s="1" t="n"/>
     </row>
-    <row r="51" ht="45.25" customHeight="1">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>KẾT LUẬN PHÂN TÍCH CUỐI CÙNG</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Mỗi kết quả phải gồm: kết luận | trạng thái | nguồn và ngày | giới hạn | bước tiếp theo</t>
+    <row r="51" ht="77.25" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Nội dung pháp lý chưa có kết luận chính thức</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Nêu câu hỏi chưa có kết luận, văn bản đã tìm, điểm mâu thuẫn, cơ quan/luật sư cần hỏi, tài liệu và thời hạn xác minh.</t>
         </is>
       </c>
       <c r="C51" s="4" t="n"/>
@@ -2912,15 +2931,15 @@
       <c r="V51" s="1" t="n"/>
       <c r="W51" s="1" t="n"/>
     </row>
-    <row r="52" ht="85.25" customHeight="1">
+    <row r="52" ht="77.25" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Đặc điểm thị trường ảnh hưởng lớn nhất đến vận hành trạm sạc</t>
+          <t>Thời gian dự phòng cần cộng thêm cho pháp lý</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Tối đa 3–5 phát hiện có bằng chứng, nêu tác động tới nhu cầu, kỹ thuật, tiến độ hoặc chi phí; tránh nhận xét chung hoặc suy diễn văn hóa.</t>
+          <t>Chỉ đưa khoảng dự phòng khi có thời hạn, trường hợp tham chiếu hoặc dữ liệu dự án. Nếu là giả định kế hoạch, phải ghi rõ phương pháp và cơ sở.</t>
         </is>
       </c>
       <c r="C52" s="4" t="n"/>
@@ -2945,15 +2964,15 @@
       <c r="V52" s="1" t="n"/>
       <c r="W52" s="1" t="n"/>
     </row>
-    <row r="53" ht="85.25" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Khả năng đáp ứng của hạ tầng điện</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Từ nguồn công khai: đơn vị điện lực, biểu giá, quy trình và yêu cầu. Khả năng cấp công suất, độ tin cậy, thời gian và chi phí tại địa điểm phải được xác nhận.</t>
+    <row r="53" ht="45.25" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>KẾT LUẬN PHÂN TÍCH CUỐI CÙNG</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Mỗi kết quả phải gồm: kết luận | trạng thái | nguồn và ngày | giới hạn | bước tiếp theo</t>
         </is>
       </c>
       <c r="C53" s="4" t="n"/>
@@ -2981,12 +3000,12 @@
     <row r="54" ht="85.25" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Thủ tục pháp lý có nguy cơ làm chậm dự án</t>
+          <t>Đặc điểm thị trường ảnh hưởng lớn nhất đến vận hành taxi điện</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Nêu 1–3 thủ tục có khả năng ảnh hưởng đường găng, căn cứ và giới hạn. Việc áp dụng cho dự án cụ thể phải được cơ quan hoặc tư vấn pháp lý xác nhận.</t>
+          <t>Tối đa 3–5 phát hiện có bằng chứng, nêu tác động tới nhu cầu, tài xế, đội xe, tiến độ hoặc chi phí; tránh nhận xét chung hoặc suy diễn văn hóa.</t>
         </is>
       </c>
       <c r="C54" s="4" t="n"/>
@@ -3014,12 +3033,12 @@
     <row r="55" ht="85.25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Nhà thầu phù hợp sơ bộ</t>
+          <t>Khả năng đáp ứng nguồn xe và sạc cho đội xe</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chọn từ đơn vị đã phân loại 'Tổng thầu turnkey' và thuộc Nhóm A ở Bảng 3B. Nếu không đủ, được đưa nhóm thấp hơn nhưng phải ghi rõ nhóm, điểm và lý do. Xếp hạng: dự án trúng thầu/chủ đầu tư xác nhận &gt; báo chí độc lập &gt; tự công bố. Đưa 1–3 đơn vị kèm bằng chứng và nội dung còn thiếu. Không coi là lựa chọn cuối trước khi kiểm tra pháp lý, tham chiếu dự án và nhận hồ sơ/báo giá.</t>
+          <t>Từ nguồn công khai: mẫu xe phân phối chính thức, bảo hành taxi, thời gian giao xe; đơn vị điện lực, biểu giá, quy trình đấu nối depot và mạng sạc dự phòng. Thời gian giao xe, công suất tại depot, độ tin cậy và chi phí cụ thể phải được nhà cung cấp/điện lực xác nhận.</t>
         </is>
       </c>
       <c r="C55" s="4" t="n"/>
@@ -3047,12 +3066,12 @@
     <row r="56" ht="85.25" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Các đối tác địa phương có thể tiếp cận</t>
+          <t>Thủ tục pháp lý có nguy cơ làm chậm khai trương</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Liệt kê theo chức năng, liên hệ chính thức và bằng chứng hoạt động. Không coi năng lực, mức độ sẵn sàng hoặc điều kiện thương mại là đã xác nhận khi chưa trao đổi trực tiếp.</t>
+          <t>Nêu 1–3 thủ tục có khả năng ảnh hưởng đường găng khai trương (giấy phép vận tải, đăng kiểm xe, depot/đấu nối), căn cứ và giới hạn. Việc áp dụng cho dự án cụ thể phải được cơ quan hoặc tư vấn pháp lý xác nhận.</t>
         </is>
       </c>
       <c r="C56" s="4" t="n"/>
@@ -3080,12 +3099,12 @@
     <row r="57" ht="85.25" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Rủi ro lớn nhất đối với tiến độ</t>
+          <t>Nhà thầu depot phù hợp sơ bộ</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Nêu rủi ro quan trọng nhất có căn cứ. Chỉ định lượng khi có dữ liệu; nếu chưa, nêu dấu hiệu cảnh báo, thông tin cần lấy, người chịu trách nhiệm và hạn xác minh.</t>
+          <t>Chỉ chọn từ đơn vị đã phân loại 'Tổng thầu turnkey' và thuộc Nhóm A ở Bảng 3B. Nếu không đủ, được đưa nhóm thấp hơn nhưng phải ghi rõ nhóm, điểm và lý do. Xếp hạng: dự án trúng thầu/chủ đầu tư xác nhận &gt; báo chí độc lập &gt; tự công bố. Đưa 1–3 đơn vị kèm bằng chứng và nội dung còn thiếu. Không coi là lựa chọn cuối trước khi kiểm tra pháp lý, tham chiếu dự án và nhận hồ sơ/báo giá.</t>
         </is>
       </c>
       <c r="C57" s="4" t="n"/>
@@ -3113,12 +3132,12 @@
     <row r="58" ht="85.25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Rủi ro lớn nhất đối với chi phí</t>
+          <t>Các đối tác địa phương có thể tiếp cận</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Nêu rủi ro quan trọng nhất có căn cứ. Khoảng tiền/% chỉ dùng khi có dữ liệu phù hợp; nếu thiếu báo giá, trình bày độ nhạy và kế hoạch lấy thông tin.</t>
+          <t>Liệt kê theo chức năng, liên hệ chính thức và bằng chứng hoạt động. Không coi năng lực, mức độ sẵn sàng hoặc điều kiện thương mại là đã xác nhận khi chưa trao đổi trực tiếp.</t>
         </is>
       </c>
       <c r="C58" s="4" t="n"/>
@@ -3143,13 +3162,21 @@
       <c r="V58" s="1" t="n"/>
       <c r="W58" s="1" t="n"/>
     </row>
-    <row r="59">
-      <c r="A59" s="1" t="n"/>
-      <c r="B59" s="1" t="n"/>
-      <c r="C59" s="1" t="n"/>
-      <c r="D59" s="1" t="n"/>
-      <c r="E59" s="1" t="n"/>
-      <c r="F59" s="1" t="n"/>
+    <row r="59" ht="85.25" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Rủi ro lớn nhất đối với tiến độ</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Nêu rủi ro quan trọng nhất có căn cứ. Chỉ định lượng khi có dữ liệu; nếu chưa, nêu dấu hiệu cảnh báo, thông tin cần lấy, người chịu trách nhiệm và hạn xác minh.</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="4" t="n"/>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
       <c r="G59" s="1" t="n"/>
       <c r="H59" s="1" t="n"/>
       <c r="I59" s="1" t="n"/>
@@ -3168,13 +3195,21 @@
       <c r="V59" s="1" t="n"/>
       <c r="W59" s="1" t="n"/>
     </row>
-    <row r="60">
-      <c r="A60" s="1" t="n"/>
-      <c r="B60" s="1" t="n"/>
-      <c r="C60" s="1" t="n"/>
-      <c r="D60" s="1" t="n"/>
-      <c r="E60" s="1" t="n"/>
-      <c r="F60" s="1" t="n"/>
+    <row r="60" ht="85.25" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Rủi ro lớn nhất đối với chi phí</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Nêu rủi ro quan trọng nhất có căn cứ. Khoảng tiền/% chỉ dùng khi có dữ liệu phù hợp; nếu thiếu báo giá, trình bày độ nhạy và kế hoạch lấy thông tin.</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
       <c r="G60" s="1" t="n"/>
       <c r="H60" s="1" t="n"/>
       <c r="I60" s="1" t="n"/>
@@ -26345,11 +26380,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26411,7 +26446,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>Mục tiêu mặc định: TỔNG THẦU TURNKEY (EPC/EC) — đơn vị tự thi công và lo trọn gói: thiết kế, vật tư/thiết bị, thi công, xin phép, thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn (§6.2 SKILL.md), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
+          <t>Mục tiêu mặc định: TỔNG THẦU XÂY DEPOT &amp; LẮP SẠC CHO ĐỘI XE (turnkey) — đơn vị tự thi công và lo trọn gói: thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc, xin phép (xây dựng, đấu nối, PCCC), thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn F1–F10 (skill contractor-search, §6.2), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
         </is>
       </c>
       <c r="B2" s="39" t="n"/>
@@ -26587,7 +26622,7 @@
       </c>
       <c r="M4" s="41" t="inlineStr">
         <is>
-          <t>Tổng điểm theo thang §6.5 của SKILL.md. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
+          <t>Tổng điểm theo thang §6.5 của skill contractor-search. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
         </is>
       </c>
       <c r="N4" s="41" t="inlineStr">
@@ -26597,7 +26632,7 @@
       </c>
       <c r="O4" s="41" t="inlineStr">
         <is>
-          <t>Khung nào tìm ra đơn vị này (F1 đấu thầu, F2 chứng chỉ năng lực, F3 điện lực, F4 ĐKKD, F5 Sở Xây dựng, F6 dự án ngược, F7 snowball, F8 ngành lân cận, F9 hiệp hội, F10 trang đại lý hãng).</t>
+          <t>Khung nào tìm ra đơn vị này (F1 đấu thầu, F2 chứng chỉ năng lực, F3 điện lực, F4 ĐKKD, F5 Sở Xây dựng, F6 dự án ngược, F7 snowball, F8 ngành lân cận, F9 hiệp hội, F10 trang đại lý hãng bộ sạc).</t>
         </is>
       </c>
       <c r="P4" s="41" t="inlineStr">
@@ -27666,7 +27701,7 @@
       </c>
       <c r="B71" s="41" t="inlineStr">
         <is>
-          <t>Kết quả lựa chọn nhà thầu (muasamcong.mpi.gov.vn) — gói EC/EPC, thiết kế và thi công, chìa khóa trao tay</t>
+          <t>Kết quả lựa chọn nhà thầu (muasamcong.mpi.gov.vn) — gói EC/EPC, thiết kế và thi công, chìa khóa trao tay: depot, bãi đỗ, nhà xưởng, hệ thống sạc đội xe, trạm biến áp</t>
         </is>
       </c>
       <c r="C71" s="45" t="n"/>
@@ -27696,7 +27731,7 @@
       </c>
       <c r="B73" s="41" t="inlineStr">
         <is>
-          <t>Đơn vị đủ điều kiện thi công đường dây và trạm biến áp (điện lực tỉnh/EVN)</t>
+          <t>Đơn vị đủ điều kiện thi công đường dây và trạm biến áp (điện lực tỉnh/EVN) — quyết định với đấu nối depot sạc</t>
         </is>
       </c>
       <c r="C73" s="45" t="n"/>
@@ -27726,7 +27761,7 @@
       </c>
       <c r="B75" s="41" t="inlineStr">
         <is>
-          <t>Sở Xây dựng / Sở Công Thương — công bố năng lực nhà thầu, giấy phép xây dựng</t>
+          <t>Sở Xây dựng / Sở Công Thương / cơ quan PCCC — công bố năng lực nhà thầu, giấy phép xây dựng, nghiệm thu PCCC</t>
         </is>
       </c>
       <c r="C75" s="45" t="n"/>
@@ -27741,7 +27776,7 @@
       </c>
       <c r="B76" s="41" t="inlineStr">
         <is>
-          <t>Dự án ngược — chủ đầu tư, ban quản lý, báo chí công bố đơn vị thi công</t>
+          <t>Dự án ngược — depot/bãi xe điện, hệ thống sạc đội xe buýt/taxi/logistics: chủ đầu tư, ban quản lý, báo chí công bố đơn vị thi công</t>
         </is>
       </c>
       <c r="C76" s="45" t="n"/>
@@ -27756,7 +27791,7 @@
       </c>
       <c r="B77" s="41" t="inlineStr">
         <is>
-          <t>Snowball — thầu phụ/liên danh nêu trong F1, F6; nhà thầu của CPO đối thủ</t>
+          <t>Snowball — thầu phụ/liên danh nêu trong F1, F6; nhà thầu đã xây depot cho hãng taxi/gọi xe đối thủ</t>
         </is>
       </c>
       <c r="C77" s="45" t="n"/>
@@ -27771,7 +27806,7 @@
       </c>
       <c r="B78" s="41" t="inlineStr">
         <is>
-          <t>Ngành lân cận — thầu điện, trạm biến áp, cơ điện M&amp;E, hạ tầng viễn thông</t>
+          <t>Ngành lân cận — thầu điện, trạm biến áp, cơ điện M&amp;E, nhà xưởng/bãi đỗ, hạ tầng viễn thông</t>
         </is>
       </c>
       <c r="C78" s="45" t="n"/>
@@ -27801,7 +27836,7 @@
       </c>
       <c r="B80" s="41" t="inlineStr">
         <is>
-          <t>Trang đại lý ủy quyền của hãng thiết bị — dùng ngược để nhận diện Cấp 2</t>
+          <t>Trang đại lý ủy quyền của hãng bộ sạc — dùng ngược để nhận diện Cấp 2</t>
         </is>
       </c>
       <c r="C80" s="45" t="n"/>
@@ -27872,7 +27907,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="33" t="inlineStr">
         <is>
-          <t>HƯỚNG DẪN SỬ DỤNG KHUNG NGHIÊN CỨU THỊ TRƯỜNG EV</t>
+          <t>HƯỚNG DẪN SỬ DỤNG KHUNG NGHIÊN CỨU THỊ TRƯỜNG TAXI ĐIỆN</t>
         </is>
       </c>
     </row>
@@ -27899,7 +27934,7 @@
       </c>
       <c r="B4" s="26" t="inlineStr">
         <is>
-          <t>Quốc gia/thị trường; thành phố/khu vực; mô hình trạm; quy mô xe; giai đoạn dự án; loại xe; địa điểm ứng viên nếu có.</t>
+          <t>Quốc gia/thị trường; thành phố/khu vực; quy mô đội xe và loại xe (mẫu xe điện dự kiến); mô hình dịch vụ (taxi, gọi xe qua app, sân bay, doanh nghiệp); giai đoạn khai trương; phương án depot và sạc; địa điểm depot ứng viên nếu có.</t>
         </is>
       </c>
       <c r="C4" s="36" t="n"/>
@@ -28011,7 +28046,7 @@
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>Chỉ kết luận ở mức phù hợp với bằng chứng. Phân biệt khu vực tiềm năng với địa điểm cụ thể; không tuyên bố “Sẵn sàng triển khai” khi thiếu xác nhận về đất, điện, pháp lý và chi phí.</t>
+          <t>Chỉ kết luận ở mức phù hợp với bằng chứng. Phân biệt khu vực tiềm năng với depot/địa điểm cụ thể; không tuyên bố “Sẵn sàng khai trương” khi thiếu xác nhận về giấy phép vận tải, nguồn xe, đất/depot, điện và chi phí.</t>
         </is>
       </c>
       <c r="C11" s="36" t="n"/>

</xml_diff>

<commit_message>
feat!: using-doox điều phối mọi yêu cầu, gộp 4 skill research, viết lại 3 tầng, bản 1.3.0
- Gộp research-method, contractor-search, competitor-research vào một
  market-research (thị trường/từ khoá, tìm nhà thầu, so đối thủ); phần
  riêng từng việc nằm trong references/, thêm quy đổi frame/chấm điểm
  nhà thầu cho thị trường ngoài Việt Nam.
- using-doox thành bộ điều phối nạp trước mọi yêu cầu Doox: 7 luật cứng
  chung, định tuyến, chuỗi skill, brief cho agent.
- Cả 12 skill viết lại theo 3 tầng: ranh giới cứng giữ nguyên, còn lại là
  mặc định có lý do mà model được lệch nếu nói rõ; bỏ thủ tục từng bước.
- reminder theo ngôn ngữ user (nhãn vi/en/fr), mail theo ngôn ngữ người nhận.
- Bỏ project-insights. Sửa description market-research sang YAML hợp lệ.

BREAKING: gọi contractor-search, competitor-research, research-method,
project-insights không còn chạy; dùng market-research / project-report.
</commit_message>
<xml_diff>
--- a/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
+++ b/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Khung báo cáo thị trường mẫu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bảng 3B - Danh sách nhà thầu" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="00 - Hướng dẫn" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khung báo cáo thị trường mẫu" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng 3B - Danh sách nhà thầu" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 - Hướng dẫn" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (F1–F10, skill contractor-search) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
+          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (F1–F10, skill market-research, references/contractor-enumeration.md) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -26446,7 +26446,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>Mục tiêu mặc định: TỔNG THẦU XÂY DEPOT &amp; LẮP SẠC CHO ĐỘI XE (turnkey) — đơn vị tự thi công và lo trọn gói: thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc, xin phép (xây dựng, đấu nối, PCCC), thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn F1–F10 (skill contractor-search, §6.2), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
+          <t>Mục tiêu mặc định: TỔNG THẦU XÂY DEPOT &amp; LẮP SẠC CHO ĐỘI XE (turnkey) — đơn vị tự thi công và lo trọn gói: thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc, xin phép (xây dựng, đấu nối, PCCC), thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn F1–F10 (skill market-research, references/contractor-enumeration.md, §6.2), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
         </is>
       </c>
       <c r="B2" s="39" t="n"/>
@@ -26622,7 +26622,7 @@
       </c>
       <c r="M4" s="41" t="inlineStr">
         <is>
-          <t>Tổng điểm theo thang §6.5 của skill contractor-search. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
+          <t>Tổng điểm theo thang §6.5 của skill market-research, references/contractor-enumeration.md. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
         </is>
       </c>
       <c r="N4" s="41" t="inlineStr">
@@ -27451,6 +27451,7 @@
       <c r="Q44" s="41" t="n"/>
       <c r="R44" s="41" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="38" t="inlineStr">
         <is>
@@ -27642,6 +27643,7 @@
       <c r="D67" s="41" t="n"/>
       <c r="E67" s="41" t="n"/>
     </row>
+    <row r="68"/>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat!: using-doox điều phối mọi yêu cầu, gộp 4 skill research, viết lại 3 tầng, bản 1.2.1
- Gộp research-method, contractor-search, competitor-research vào một
  market-research (thị trường/từ khoá, tìm nhà thầu, so đối thủ); phần
  riêng từng việc nằm trong references/, thêm quy đổi frame/chấm điểm
  nhà thầu cho thị trường ngoài Việt Nam.
- using-doox thành bộ điều phối nạp trước mọi yêu cầu Doox: 7 luật cứng
  chung, định tuyến, chuỗi skill, brief cho agent.
- Cả 12 skill viết lại theo 3 tầng: ranh giới cứng giữ nguyên, còn lại là
  mặc định có lý do mà model được lệch nếu nói rõ; bỏ thủ tục từng bước.
- reminder theo ngôn ngữ user (nhãn vi/en/fr), mail theo ngôn ngữ người nhận.
- Bỏ project-insights. Sửa description market-research sang YAML hợp lệ.

BREAKING: gọi contractor-search, competitor-research, research-method,
project-insights không còn chạy; dùng market-research / project-report.
</commit_message>
<xml_diff>
--- a/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
+++ b/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Khung báo cáo thị trường mẫu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bảng 3B - Danh sách nhà thầu" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="00 - Hướng dẫn" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khung báo cáo thị trường mẫu" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng 3B - Danh sách nhà thầu" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 - Hướng dẫn" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (F1–F10, skill contractor-search) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
+          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (F1–F10, skill market-research, references/contractor-enumeration.md) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -26446,7 +26446,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>Mục tiêu mặc định: TỔNG THẦU XÂY DEPOT &amp; LẮP SẠC CHO ĐỘI XE (turnkey) — đơn vị tự thi công và lo trọn gói: thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc, xin phép (xây dựng, đấu nối, PCCC), thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn F1–F10 (skill contractor-search, §6.2), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
+          <t>Mục tiêu mặc định: TỔNG THẦU XÂY DEPOT &amp; LẮP SẠC CHO ĐỘI XE (turnkey) — đơn vị tự thi công và lo trọn gói: thiết kế, xây dựng depot/bãi đỗ, hạ tầng điện và trạm biến áp, cung cấp và lắp đặt bộ sạc, xin phép (xây dựng, đấu nối, PCCC), thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn F1–F10 (skill market-research, references/contractor-enumeration.md, §6.2), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
         </is>
       </c>
       <c r="B2" s="39" t="n"/>
@@ -26622,7 +26622,7 @@
       </c>
       <c r="M4" s="41" t="inlineStr">
         <is>
-          <t>Tổng điểm theo thang §6.5 của skill contractor-search. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
+          <t>Tổng điểm theo thang §6.5 của skill market-research, references/contractor-enumeration.md. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
         </is>
       </c>
       <c r="N4" s="41" t="inlineStr">
@@ -27451,6 +27451,7 @@
       <c r="Q44" s="41" t="n"/>
       <c r="R44" s="41" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="38" t="inlineStr">
         <is>
@@ -27642,6 +27643,7 @@
       <c r="D67" s="41" t="n"/>
       <c r="E67" s="41" t="n"/>
     </row>
+    <row r="68"/>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="38" t="inlineStr">
         <is>

</xml_diff>